<commit_message>
feat: complete v4 sequence template with flowcharts, update and deploy mobile app, launch servers
</commit_message>
<xml_diff>
--- a/projects/plc-monitoring-v1/GMS_자동진행_시퀀스_표준템플릿_v4.xlsx
+++ b/projects/plc-monitoring-v1/GMS_자동진행_시퀀스_표준템플릿_v4.xlsx
@@ -24,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -87,11 +87,28 @@
     <font>
       <name val="맑은 고딕"/>
       <b val="1"/>
+      <color rgb="002563EB"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
       <color rgb="00047857"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Consolas"/>
+      <color rgb="001E293B"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="00B45309"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="13">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -164,8 +181,26 @@
         <bgColor rgb="00047857"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00334155"/>
+        <bgColor rgb="00334155"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EFF6FF"/>
+        <bgColor rgb="00EFF6FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F1F5F9"/>
+        <bgColor rgb="00F1F5F9"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -187,11 +222,67 @@
         <color rgb="00CBD5E1"/>
       </bottom>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="003B82F6"/>
+      </left>
+      <right style="medium">
+        <color rgb="003B82F6"/>
+      </right>
+      <top style="medium">
+        <color rgb="003B82F6"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="003B82F6"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="0010B981"/>
+      </left>
+      <right style="medium">
+        <color rgb="0010B981"/>
+      </right>
+      <top style="medium">
+        <color rgb="0010B981"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="0010B981"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="0064748B"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00F59E0B"/>
+      </left>
+      <right style="medium">
+        <color rgb="00F59E0B"/>
+      </right>
+      <top style="medium">
+        <color rgb="00F59E0B"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00F59E0B"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -254,7 +345,28 @@
     <xf numFmtId="0" fontId="9" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="15" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -644,7 +756,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>본 시트는 GMS 35개 전체 컬럼 문법, 타임차트/플로우차트 렌더링 엔진 연동 규칙, 6대 실무 상황별 예제 시트 바로가기를 완벽 제공합니다.</t>
+          <t>본 시트는 GMS 35개 전체 컬럼 문법, Mermaid 공식 플로우차트 기법, 6대 실무 상황별 예제 시트 바로가기를 완벽 제공합니다.</t>
         </is>
       </c>
     </row>
@@ -795,7 +907,7 @@
       <c r="D12" s="7" t="n"/>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>필요한 밸브만 O/C 입력하고, 빈칸(공백)은 이전 상태를 유지하는 방법 학습</t>
+          <t>필요한 밸브만 O/C 입력하고, 빈칸(공백)은 이전 상태 유지 ➔ 시트 하단 비주얼/Mermaid 플로우차트 제공</t>
         </is>
       </c>
       <c r="F12" s="7" t="n"/>
@@ -820,7 +932,7 @@
       <c r="D13" s="7" t="n"/>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>120초 설정했으나 0.5 Torr 도달 시 5초 만에 즉시 다음 스텝 통과하는 방법 학습</t>
+          <t>120초 설정했으나 0.5 Torr 도달 시 5초 만에 즉시 다음 스텝 패스 ➔ Early Pass 분기 플로우차트 제공</t>
         </is>
       </c>
       <c r="F13" s="7" t="n"/>
@@ -845,7 +957,7 @@
       <c r="D14" s="7" t="n"/>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>진행방식 '확인' 설정 시 작업자가 버튼을 누를 때까지 정지 대기하는 방법 학습</t>
+          <t>진행방식 '확인' 설정 시 작업자가 버튼 누를 때까지 정지 대기 ➔ 수동 승인 대기 플로우차트 제공</t>
         </is>
       </c>
       <c r="F14" s="7" t="n"/>
@@ -870,7 +982,7 @@
       <c r="D15" s="7" t="n"/>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>O+2, O+4 문법을 사용하여 밸브를 2초, 4초 간격으로 순차 개폐하는 방법 학습</t>
+          <t>O+2, O+4 문법을 사용하여 밸브를 2초, 4초 간격으로 순차 개폐 ➔ 시차 제어 플로우차트 제공</t>
         </is>
       </c>
       <c r="F15" s="7" t="n"/>
@@ -895,7 +1007,7 @@
       <c r="D16" s="7" t="n"/>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>★개선: 진행횟수 &gt;= 3 판정 시 Next Step, 미달 시 Alarm Goto로 복귀하는 정상 루프 학습</t>
+          <t>진행횟수 &gt;= 3 판정 시 Next Step, 미달 시 Alarm Goto로 복귀 ➔ 루프백(Loop-back) 플로우차트 제공</t>
         </is>
       </c>
       <c r="F16" s="7" t="n"/>
@@ -920,7 +1032,7 @@
       <c r="D17" s="7" t="n"/>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>★신설: CAPTURE 문법으로 초기압력 저장 후 :CAPOFFSET으로 허용변동량 이내인지 검사</t>
+          <t>CAPTURE 문법으로 초기압력 저장 후 :CAPOFFSET으로 누출량 판정 ➔ 정밀 검사 플로우차트 제공</t>
         </is>
       </c>
       <c r="F17" s="7" t="n"/>
@@ -945,7 +1057,7 @@
       <c r="D18" s="7" t="n"/>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>실제 현장 가스 캐비닛 장비에 즉시 업로드 가능한 완전한 시퀀스 양식 학습</t>
+          <t>현장 가스 캐비닛 장비에 즉시 업로드 가능한 완전한 시퀀스 ➔ 전 공정 종합 Mermaid 플로우차트 탑재</t>
         </is>
       </c>
       <c r="F18" s="7" t="n"/>
@@ -1885,7 +1997,7 @@
     <row r="50" ht="28" customHeight="1">
       <c r="A50" s="15" t="inlineStr">
         <is>
-          <t>4. ★ 시퀀스 차트(Time Chart &amp; Flow Chart) 렌더링 엔진 연동 가이드</t>
+          <t>4. ★ 플로우차트(Mermaid 기법) 및 시퀀스 타임차트 연동 가이드</t>
         </is>
       </c>
     </row>
@@ -1907,29 +2019,29 @@
       </c>
       <c r="D51" s="16" t="inlineStr">
         <is>
-          <t>차트 렌더링 시각화 규칙 (주의사항)</t>
+          <t>공식 Mermaid 및 렌더링 규칙</t>
         </is>
       </c>
     </row>
     <row r="52" ht="28" customHeight="1">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>타임차트 (Gantt)</t>
+          <t>플로우차트 (공식 기법)</t>
         </is>
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>공백(빈칸) 셀 처리</t>
+          <t>Mermaid.js (flowchart TD)</t>
         </is>
       </c>
       <c r="C52" s="6" t="inlineStr">
         <is>
-          <t>이전 스텝의 밸브 개폐 상태를 누적 상속(Carry-forward)</t>
+          <t>프로젝트 표준 문서([Q-004], [Q-013], [Q-014]) 공식 채택 기법</t>
         </is>
       </c>
       <c r="D52" s="6" t="inlineStr">
         <is>
-          <t>★빈칸을 CLOSE(0)로 그리면 차트 선이 끊어집니다! 직전 스텝의 ON/OFF 상태를 그대로 연장하여 연속된 바로 그려야 합니다.</t>
+          <t>★모든 예제 시트 하단에 비주얼 블록 다이어그램과 Mermaid 소스코드가 1:1로 함께 탑재되어 있습니다.</t>
         </is>
       </c>
       <c r="E52" s="7" t="n"/>
@@ -1939,22 +2051,22 @@
     <row r="53" ht="28" customHeight="1">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>타임차트 (Gantt)</t>
+          <t>플로우차트 (Mermaid)</t>
         </is>
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>지연 개폐 (O+n, C+n)</t>
+          <t>정상 진행선 (실선 화살표)</t>
         </is>
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
-          <t>스텝 시작점(T0)으로부터 +n초 시점에 상태 전이 발생</t>
+          <t>Next Step 지정 시 S/No ➔ Next Step, 미지정 시 S/No ➔ S/No+1</t>
         </is>
       </c>
       <c r="D53" s="6" t="inlineStr">
         <is>
-          <t>스텝 전체 시간 바 안에서 +n초 오프셋 지점에 색상 반전(Rising/Falling Edge) 마커를 표시해야 합니다.</t>
+          <t>S1 --&gt; S2 (녹색/파랑 실선 화살표로 연결)</t>
         </is>
       </c>
       <c r="E53" s="7" t="n"/>
@@ -1964,22 +2076,22 @@
     <row r="54" ht="28" customHeight="1">
       <c r="A54" s="5" t="inlineStr">
         <is>
-          <t>타임차트 (Gantt)</t>
+          <t>플로우차트 (Mermaid)</t>
         </is>
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>조기통과 (Early Pass)</t>
+          <t>루프 반복선 (Loop-back)</t>
         </is>
       </c>
       <c r="C54" s="6" t="inlineStr">
         <is>
-          <t>Time(Sec) 전체를 점선 바로 표시하고, 통과 예상 시점을 마킹</t>
+          <t>Alarm Monitoring='진행횟수' 조건 불만족 시 Alarm Goto로 복귀</t>
         </is>
       </c>
       <c r="D54" s="6" t="inlineStr">
         <is>
-          <t>조기통과 조건 충족 시 실제 시간은 단축되므로, 예상 최대 시간(점선)과 최소 보장 시간(실선)을 구분하여 표시합니다.</t>
+          <t>S3 -- '거짓(미달) [Alarm Goto: 2]' --&gt; S2 (주황/점선 루프백)</t>
         </is>
       </c>
       <c r="E54" s="7" t="n"/>
@@ -1989,22 +2101,22 @@
     <row r="55" ht="28" customHeight="1">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t>플로우차트 (Flow)</t>
+          <t>플로우차트 (Mermaid)</t>
         </is>
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>정상 진행선</t>
+          <t>비상 알람선 (Alarm)</t>
         </is>
       </c>
       <c r="C55" s="6" t="inlineStr">
         <is>
-          <t>Next Step이 공백이면 S/No.+1로 이동, 지정 시 Next Step으로 점프</t>
+          <t>센서 감시 조건 불만족 시 Alarm Goto 번호로 비상 점프</t>
         </is>
       </c>
       <c r="D55" s="6" t="inlineStr">
         <is>
-          <t>초록색 실선 화살표로 연결합니다.</t>
+          <t>S2 -- '알람 발생 [Goto 99]' --&gt; S99['비상 정지']:::alarmNode</t>
         </is>
       </c>
       <c r="E55" s="7" t="n"/>
@@ -2014,22 +2126,22 @@
     <row r="56" ht="28" customHeight="1">
       <c r="A56" s="5" t="inlineStr">
         <is>
-          <t>플로우차트 (Flow)</t>
+          <t>플로우차트 (Mermaid)</t>
         </is>
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>루프 반복선</t>
+          <t>수동 확인 대기 (ACK)</t>
         </is>
       </c>
       <c r="C56" s="6" t="inlineStr">
         <is>
-          <t>'진행횟수' 조건 불만족 시 Alarm Goto 번호로 루프백 점프</t>
+          <t>진행방식 = '확인(ack)'</t>
         </is>
       </c>
       <c r="D56" s="6" t="inlineStr">
         <is>
-          <t>주황색/파란색 점선 화살표로 이전 스텝에 되돌아가는 루프백(Loop-back) 연결을 표시하고 'N회 반복' 배지를 표시합니다.</t>
+          <t>S2{'작업자 육안 확인 대기'} -- '[확인] 버튼 클릭' --&gt; S3</t>
         </is>
       </c>
       <c r="E56" s="7" t="n"/>
@@ -2039,22 +2151,22 @@
     <row r="57" ht="28" customHeight="1">
       <c r="A57" s="5" t="inlineStr">
         <is>
-          <t>플로우차트 (Flow)</t>
+          <t>타임차트 (Gantt)</t>
         </is>
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>비상 알람선</t>
+          <t>공백(빈칸) 셀 처리</t>
         </is>
       </c>
       <c r="C57" s="6" t="inlineStr">
         <is>
-          <t>센서 조건 불만족 시 Alarm Goto 번호로 비상 점프</t>
+          <t>이전 스텝의 밸브 개폐 상태를 누적 상속(Carry-forward)</t>
         </is>
       </c>
       <c r="D57" s="6" t="inlineStr">
         <is>
-          <t>빨간색 실선 화살표로 비상 대응 스텝(Step 99)으로 연결하고 경고 아이콘을 표시합니다.</t>
+          <t>빈칸을 CLOSE(0)로 그리지 않고 이전 ON/OFF 상태를 연장하여 연속된 바로 렌더링</t>
         </is>
       </c>
       <c r="E57" s="7" t="n"/>
@@ -2064,22 +2176,22 @@
     <row r="58" ht="28" customHeight="1">
       <c r="A58" s="5" t="inlineStr">
         <is>
-          <t>플로우차트 (Flow)</t>
+          <t>타임차트 (Gantt)</t>
         </is>
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>수동 확인 대기</t>
+          <t>지연 개폐 (O+n, C+n)</t>
         </is>
       </c>
       <c r="C58" s="6" t="inlineStr">
         <is>
-          <t>진행방식 = '확인(ack)'</t>
+          <t>스텝 시작점(T0)으로부터 +n초 시점에 상태 전이 발생</t>
         </is>
       </c>
       <c r="D58" s="6" t="inlineStr">
         <is>
-          <t>단계 블록 옆에 손가락/버튼 아이콘을 띄워 작업자 수동 승인 후 진행됨을 직관적으로 표시합니다.</t>
+          <t>스텝 전체 시간 바 안에서 +n초 오프셋 지점에 Rising/Falling Edge 마커 표시</t>
         </is>
       </c>
       <c r="E58" s="7" t="n"/>
@@ -2153,7 +2265,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF7"/>
+  <dimension ref="A1:AF28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2603,14 +2715,145 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10" ht="28" customHeight="1">
+      <c r="A10" s="24" t="inlineStr">
+        <is>
+          <t>📊 [공정 시퀀스 플로우차트 - 비주얼 블록 다이어그램 &amp; 공식 Mermaid 기법]</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>🎨 비주얼 공정 흐름도 (Visual Step Flowchart)</t>
+        </is>
+      </c>
+      <c r="M11" s="25" t="inlineStr">
+        <is>
+          <t>📜 공식 Mermaid 기법 소스 코드 (flowchart TD - 복사용)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="26" customHeight="1">
+      <c r="B12" s="26" t="inlineStr">
+        <is>
+          <t>▶ [Step 1] 전 밸브 안전 Close | 5초 대기 (VN1=C, VN2=C, PNV=C, HPV=C)</t>
+        </is>
+      </c>
+      <c r="M12" s="27" t="inlineStr">
+        <is>
+          <t>```mermaid
+flowchart TD
+    classDef startNode fill:#1e40af,stroke:#1e3a8a,color:#fff,font-weight:bold
+    classDef procNode fill:#eff6ff,stroke:#3b82f6,color:#1e3a8a,font-weight:bold
+    classDef passNode fill:#d1fae5,stroke:#10b981,color:#047857,font-weight:bold
+    Start(["[공정 시작] 예제1_단순개폐"]):::startNode
+    S1["[Step 1] 전 밸브 안전 Close (5초)&lt;br&gt;• VN1=C, VN2=C, PNV=C, HPV=C"]:::procNode
+    S2["[Step 2] 질소 가스 공급 개방 (30초)&lt;br&gt;• VN1=O, PNV=O (나머지 밸브 빈칸=상태유지)"]:::procNode
+    S3["[Step 3] 질소 차단 및 대기 (10초)&lt;br&gt;• VN1=C, PNV=C 닫고 안정화 대기"]:::procNode
+    EndNode(["[공정 완료] 정상 종료"]):::passNode
+    Start --&gt; S1
+    S1 --&gt;|5초 카운트다운 완료| S2
+    S2 --&gt;|30초 카운트다운 완료| S3
+    S3 --&gt;|10초 카운트다운 완료| EndNode
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="B13" s="28" t="inlineStr">
+        <is>
+          <t>│</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="B14" s="28" t="inlineStr">
+        <is>
+          <t>▼ (5초 경과 후 자동 진행)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="26" customHeight="1">
+      <c r="B15" s="26" t="inlineStr">
+        <is>
+          <t>▶ [Step 2] 질소 가스 공급 개방 | 30초 유지 (VN1=O, PNV=O / 공백 밸브 상태유지)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="B16" s="28" t="inlineStr">
+        <is>
+          <t>│</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="B17" s="28" t="inlineStr">
+        <is>
+          <t>▼ (30초 경과 후 자동 진행)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="26" customHeight="1">
+      <c r="B18" s="26" t="inlineStr">
+        <is>
+          <t>▶ [Step 3] 질소 차단 및 대기 | 10초 안정화 (VN1=C, PNV=C)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="B19" s="28" t="inlineStr">
+        <is>
+          <t>│</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="B20" s="28" t="inlineStr">
+        <is>
+          <t>▼ (10초 경과 후 정상 종료)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="26" customHeight="1">
+      <c r="B21" s="29" t="inlineStr">
+        <is>
+          <t>★ [공정 정상 완료] | 전 밸브 안전 Close 및 다음 서브시퀀스 인계</t>
+        </is>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="20">
+    <mergeCell ref="A10:AF10"/>
+    <mergeCell ref="M3:Y3"/>
+    <mergeCell ref="B14:J14"/>
+    <mergeCell ref="A11:K11"/>
+    <mergeCell ref="B17:J17"/>
+    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="B13:J13"/>
     <mergeCell ref="A2:L2"/>
+    <mergeCell ref="B19:J19"/>
     <mergeCell ref="A1:AF1"/>
-    <mergeCell ref="M3:Y3"/>
+    <mergeCell ref="M11:AF11"/>
+    <mergeCell ref="M2:AF2"/>
+    <mergeCell ref="B15:J15"/>
+    <mergeCell ref="M12:AF28"/>
+    <mergeCell ref="B20:J20"/>
+    <mergeCell ref="B16:J16"/>
     <mergeCell ref="Z3:AF3"/>
-    <mergeCell ref="M2:AF2"/>
-    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="B18:J18"/>
+    <mergeCell ref="B12:J12"/>
+    <mergeCell ref="B21:J21"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
@@ -2625,7 +2868,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF7"/>
+  <dimension ref="A1:AF32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -2991,7 +3234,7 @@
           <t>0.5</t>
         </is>
       </c>
-      <c r="AC6" s="24" t="inlineStr">
+      <c r="AC6" s="30" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -3075,14 +3318,153 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10" ht="28" customHeight="1">
+      <c r="A10" s="24" t="inlineStr">
+        <is>
+          <t>📊 [공정 시퀀스 플로우차트 - 비주얼 블록 다이어그램 &amp; 공식 Mermaid 기법]</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>🎨 비주얼 공정 흐름도 (Visual Step Flowchart)</t>
+        </is>
+      </c>
+      <c r="M11" s="25" t="inlineStr">
+        <is>
+          <t>📜 공식 Mermaid 기법 소스 코드 (flowchart TD - 복사용)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="26" customHeight="1">
+      <c r="B12" s="26" t="inlineStr">
+        <is>
+          <t>▶ [Step 1] 진공 라인 밸브 개방 | 5초 대기 (HPV=O)</t>
+        </is>
+      </c>
+      <c r="M12" s="27" t="inlineStr">
+        <is>
+          <t>```mermaid
+flowchart TD
+    classDef startNode fill:#1e40af,stroke:#1e3a8a,color:#fff,font-weight:bold
+    classDef procNode fill:#eff6ff,stroke:#3b82f6,color:#1e3a8a,font-weight:bold
+    classDef condNode fill:#fef3c7,stroke:#f59e0b,color:#b45309,font-weight:bold
+    classDef passNode fill:#d1fae5,stroke:#10b981,color:#047857,font-weight:bold
+    classDef alarmNode fill:#fee2e2,stroke:#ef4444,color:#b91c1c,font-weight:bold
+    Start(["[공정 시작] 예제2_조기통과"]):::startNode
+    S1["[Step 1] 진공 라인 밸브 개방 (5초)&lt;br&gt;• HPV=O"]:::procNode
+    S2["[Step 2] 고진공 배기 120초 대기&lt;br&gt;• 감시: VPT &lt;= 0.5 Torr&lt;br&gt;• 조기통과(Early Pass) = Y"]:::condNode
+    S3["[Step 3] 진공 유지 및 다음 공정 (10초)&lt;br&gt;• HPV=C 닫고 대기"]:::procNode
+    S99["[Step 99] 비상 정지 (Alarm Seq 1)&lt;br&gt;• 120초 내 진공 미도달 (누설 의심)"]:::alarmNode
+    EndNode(["[공정 완료]"]):::passNode
+    Start --&gt; S1
+    S1 --&gt; S2
+    S2 -- "VPT &lt;= 0.5 Torr 도달&lt;br&gt;(남은 시간 무시하고 즉시 통과!)" --&gt; S3
+    S2 -- "120초 경과할 때까지 미도달&lt;br&gt;[Alarm Goto: 99]" --&gt; S99
+    S3 --&gt; EndNode
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="B13" s="28" t="inlineStr">
+        <is>
+          <t>│</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="B14" s="28" t="inlineStr">
+        <is>
+          <t>▼ (5초 경과)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="26" customHeight="1">
+      <c r="B15" s="26" t="inlineStr">
+        <is>
+          <t>▶ [Step 2] 고진공 배기 (조기통과 Y) | Time: 120초 / 목표: VPT &lt;= 0.5 Torr</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="B16" s="28" t="inlineStr">
+        <is>
+          <t>├─ [조건 충족: VPT &lt;= 0.5 Torr] ➔ ★ 조기통과 (Early Pass, 즉시 진행)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="B17" s="28" t="inlineStr">
+        <is>
+          <t>└─ [조건 미달: 120초 경과] ➔ ▲ 비상 알람 발생 (Alarm Goto: 99 / Alarm Seq 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="26" customHeight="1">
+      <c r="B18" s="26" t="inlineStr">
+        <is>
+          <t>▶ [Step 3] 진공 유지 및 다음 공정 | 10초 대기 (HPV=C 닫힘)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="B19" s="28" t="inlineStr">
+        <is>
+          <t>│</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="B20" s="28" t="inlineStr">
+        <is>
+          <t>▼</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="26" customHeight="1">
+      <c r="B21" s="29" t="inlineStr">
+        <is>
+          <t>★ [공정 정상 완료] | 진공 배기 완료 후 안전 종료</t>
+        </is>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="20">
+    <mergeCell ref="A10:AF10"/>
+    <mergeCell ref="M3:Y3"/>
+    <mergeCell ref="B14:J14"/>
+    <mergeCell ref="A11:K11"/>
+    <mergeCell ref="B17:J17"/>
+    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="B13:J13"/>
     <mergeCell ref="A2:L2"/>
+    <mergeCell ref="B19:J19"/>
     <mergeCell ref="A1:AF1"/>
-    <mergeCell ref="M3:Y3"/>
+    <mergeCell ref="M11:AF11"/>
+    <mergeCell ref="M2:AF2"/>
+    <mergeCell ref="B15:J15"/>
+    <mergeCell ref="B20:J20"/>
+    <mergeCell ref="M12:AF32"/>
+    <mergeCell ref="B16:J16"/>
     <mergeCell ref="Z3:AF3"/>
-    <mergeCell ref="M2:AF2"/>
-    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="B18:J18"/>
+    <mergeCell ref="B12:J12"/>
+    <mergeCell ref="B21:J21"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
@@ -3097,7 +3479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF7"/>
+  <dimension ref="A1:AF29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -3535,14 +3917,147 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10" ht="28" customHeight="1">
+      <c r="A10" s="24" t="inlineStr">
+        <is>
+          <t>📊 [공정 시퀀스 플로우차트 - 비주얼 블록 다이어그램 &amp; 공식 Mermaid 기법]</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>🎨 비주얼 공정 흐름도 (Visual Step Flowchart)</t>
+        </is>
+      </c>
+      <c r="M11" s="25" t="inlineStr">
+        <is>
+          <t>📜 공식 Mermaid 기법 소스 코드 (flowchart TD - 복사용)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="26" customHeight="1">
+      <c r="B12" s="26" t="inlineStr">
+        <is>
+          <t>▶ [Step 1] 시험 압력 가압 진행 | 20초 주입 (VN1=O, PNV=O)</t>
+        </is>
+      </c>
+      <c r="M12" s="27" t="inlineStr">
+        <is>
+          <t>```mermaid
+flowchart TD
+    classDef startNode fill:#1e40af,stroke:#1e3a8a,color:#fff,font-weight:bold
+    classDef procNode fill:#eff6ff,stroke:#3b82f6,color:#1e3a8a,font-weight:bold
+    classDef ackNode fill:#fef3c7,stroke:#f59e0b,color:#b45309,font-weight:bold
+    classDef passNode fill:#d1fae5,stroke:#10b981,color:#047857,font-weight:bold
+    Start(["[공정 시작] 예제3_수동확인"]):::startNode
+    S1["[Step 1] 시험 압력 가압 진행 (20초)&lt;br&gt;• VN1=O, PNV=O (가스 주입)"]:::procNode
+    S2{"[Step 2] 작업자 육안 확인 대기&lt;br&gt;• 진행방식 = 확인 (ACK)&lt;br&gt;• 화면 [확인] 클릭 전까지 무한 대기"}:::ackNode
+    S3["[Step 3] 가압 해제 및 배기 (10초)&lt;br&gt;• HPV=O (배기 밸브 Open)"]:::procNode
+    EndNode(["[공정 완료]"]):::passNode
+    Start --&gt; S1
+    S1 --&gt;|20초 가압 완료| S2
+    S2 -- "작업자가 HMI 화면의&lt;br&gt;[확인(ACK)] 버튼 클릭" --&gt; S3
+    S3 --&gt;|10초 배기 완료| EndNode
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="B13" s="28" t="inlineStr">
+        <is>
+          <t>│</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="B14" s="28" t="inlineStr">
+        <is>
+          <t>▼</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="26" customHeight="1">
+      <c r="B15" s="31" t="inlineStr">
+        <is>
+          <t>◆ [Step 2] 작업자 육안 확인 대기 (ACK) | 진행방식 = 확인 / Time = 0초 무한 대기</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="B16" s="28" t="inlineStr">
+        <is>
+          <t>│  (현장 게이지 확인 후 화면의 [확인] 버튼 클릭)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="B17" s="28" t="inlineStr">
+        <is>
+          <t>▼</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="26" customHeight="1">
+      <c r="B18" s="26" t="inlineStr">
+        <is>
+          <t>▶ [Step 3] 가압 해제 및 완료 | 10초 배기 (HPV=O)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="B19" s="28" t="inlineStr">
+        <is>
+          <t>│</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="B20" s="28" t="inlineStr">
+        <is>
+          <t>▼</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="26" customHeight="1">
+      <c r="B21" s="29" t="inlineStr">
+        <is>
+          <t>★ [공정 정상 완료] | 작업자 확인 승인 후 배기 완료</t>
+        </is>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="20">
+    <mergeCell ref="A10:AF10"/>
+    <mergeCell ref="M3:Y3"/>
+    <mergeCell ref="B14:J14"/>
+    <mergeCell ref="A11:K11"/>
+    <mergeCell ref="B17:J17"/>
+    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="B13:J13"/>
     <mergeCell ref="A2:L2"/>
+    <mergeCell ref="B19:J19"/>
     <mergeCell ref="A1:AF1"/>
-    <mergeCell ref="M3:Y3"/>
+    <mergeCell ref="M11:AF11"/>
+    <mergeCell ref="M2:AF2"/>
+    <mergeCell ref="B15:J15"/>
+    <mergeCell ref="B20:J20"/>
+    <mergeCell ref="B16:J16"/>
     <mergeCell ref="Z3:AF3"/>
-    <mergeCell ref="M2:AF2"/>
-    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="B18:J18"/>
+    <mergeCell ref="M12:AF29"/>
+    <mergeCell ref="B12:J12"/>
+    <mergeCell ref="B21:J21"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
@@ -3557,7 +4072,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF6"/>
+  <dimension ref="A1:AF31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3938,14 +4453,132 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9" ht="28" customHeight="1">
+      <c r="A9" s="24" t="inlineStr">
+        <is>
+          <t>📊 [공정 시퀀스 플로우차트 - 비주얼 블록 다이어그램 &amp; 공식 Mermaid 기법]</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>🎨 비주얼 공정 흐름도 (Visual Step Flowchart)</t>
+        </is>
+      </c>
+      <c r="M10" s="25" t="inlineStr">
+        <is>
+          <t>📜 공식 Mermaid 기법 소스 코드 (flowchart TD - 복사용)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="26" customHeight="1">
+      <c r="B11" s="26" t="inlineStr">
+        <is>
+          <t>▶ [Step 1] 충격 방지 순차 지연 개방 | 총 15초 유지 (T+0s: VN2=O ➔ T+2s: LPV=O ➔ T+4s: HPIV=O)</t>
+        </is>
+      </c>
+      <c r="M11" s="27" t="inlineStr">
+        <is>
+          <t>```mermaid
+flowchart TD
+    classDef startNode fill:#1e40af,stroke:#1e3a8a,color:#fff,font-weight:bold
+    classDef procNode fill:#eff6ff,stroke:#3b82f6,color:#1e3a8a,font-weight:bold
+    classDef passNode fill:#d1fae5,stroke:#10b981,color:#047857,font-weight:bold
+    Start(["[공정 시작] 예제4_지연개폐"]):::startNode
+    subgraph Step1 ["Step 1: 충격 방지 순차 지연 개방 (총 15초)"]
+        T0["T+0초: VN2 즉시 Open (O)"] --&gt; T2["T+2초: LPV 지연 Open (O+2)"]
+        T2 --&gt; T4["T+4초: HPIV 지연 Open (O+4)"]
+    end
+    subgraph Step2 ["Step 2: 순차 지연 닫힘 제어 (총 10초)"]
+        C0["T+0초: VN2 즉시 Close (C)"] --&gt; C2["T+2초: LPV 지연 Close (C+2)"]
+        C2 --&gt; C3["T+3초: HPIV 지연 Close (C+3)"]
+    end
+    EndNode(["[공정 완료]"]):::passNode
+    Start --&gt; Step1
+    Step1 --&gt;|15초 완료| Step2
+    Step2 --&gt;|10초 완료| EndNode
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="B12" s="28" t="inlineStr">
+        <is>
+          <t>│</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="B13" s="28" t="inlineStr">
+        <is>
+          <t>▼ (15초 경과)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="26" customHeight="1">
+      <c r="B14" s="26" t="inlineStr">
+        <is>
+          <t>▶ [Step 2] 순차 지연 닫힘 제어 | 총 10초 유지 (T+0s: VN2=C ➔ T+2s: LPV=C ➔ T+3s: HPIV=C)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="B15" s="28" t="inlineStr">
+        <is>
+          <t>│</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="B16" s="28" t="inlineStr">
+        <is>
+          <t>▼ (10초 경과)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="26" customHeight="1">
+      <c r="B17" s="29" t="inlineStr">
+        <is>
+          <t>★ [공정 정상 완료] | 배관 충격 없이 순차 개폐 완료</t>
+        </is>
+      </c>
+    </row>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="17">
+    <mergeCell ref="B15:J15"/>
     <mergeCell ref="A2:L2"/>
+    <mergeCell ref="B11:J11"/>
     <mergeCell ref="A1:AF1"/>
+    <mergeCell ref="B16:J16"/>
     <mergeCell ref="M3:Y3"/>
     <mergeCell ref="Z3:AF3"/>
+    <mergeCell ref="B14:J14"/>
+    <mergeCell ref="B17:J17"/>
+    <mergeCell ref="A9:AF9"/>
+    <mergeCell ref="A10:K10"/>
     <mergeCell ref="M2:AF2"/>
     <mergeCell ref="A3:L3"/>
+    <mergeCell ref="B13:J13"/>
+    <mergeCell ref="M11:AF31"/>
+    <mergeCell ref="B12:J12"/>
+    <mergeCell ref="M10:AF10"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
@@ -3960,7 +4593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF8"/>
+  <dimension ref="A1:AF33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="37" customWidth="1" min="1" max="1"/>
@@ -4497,14 +5130,174 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11" ht="28" customHeight="1">
+      <c r="A11" s="24" t="inlineStr">
+        <is>
+          <t>📊 [공정 시퀀스 플로우차트 - 비주얼 블록 다이어그램 &amp; 공식 Mermaid 기법]</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>🎨 비주얼 공정 흐름도 (Visual Step Flowchart)</t>
+        </is>
+      </c>
+      <c r="M12" s="25" t="inlineStr">
+        <is>
+          <t>📜 공식 Mermaid 기법 소스 코드 (flowchart TD - 복사용)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="26" customHeight="1">
+      <c r="B13" s="26" t="inlineStr">
+        <is>
+          <t>▶ [Step 1] 루프 준비 - 밸브 초기화 | 5초 대기 (전 밸브 Close)</t>
+        </is>
+      </c>
+      <c r="M13" s="27" t="inlineStr">
+        <is>
+          <t>```mermaid
+flowchart TD
+    classDef startNode fill:#1e40af,stroke:#1e3a8a,color:#fff,font-weight:bold
+    classDef procNode fill:#eff6ff,stroke:#3b82f6,color:#1e3a8a,font-weight:bold
+    classDef condNode fill:#fef3c7,stroke:#f59e0b,color:#b45309,font-weight:bold
+    classDef passNode fill:#d1fae5,stroke:#10b981,color:#047857,font-weight:bold
+    Start(["[공정 시작] 예제5_반복루프"]):::startNode
+    S1["[Step 1] 루프 준비 - 전 밸브 Close (5초)"]:::procNode
+    S2["[Step 2] 퍼지 가스 가압 (10초)&lt;br&gt;• VN1=O, PNV=O&lt;br&gt;★ 루프 시작점 (Alarm Goto 목적지)"]:::procNode
+    S3{"[Step 3] 배기 진행 (15초)&lt;br&gt;판정: 진행횟수 &gt;= 3 ?"}:::condNode
+    S4["[Step 4] 3회 반복 완료 및 정상 종료 (5초)&lt;br&gt;• 전 밸브 Close"]:::procNode
+    EndNode(["[공정 완료] 정상 종료"]):::passNode
+    Start --&gt; S1
+    S1 --&gt; S2
+    S2 --&gt; S3
+    S3 -- "거짓 (아직 1~2회차)&lt;br&gt;[Alarm Goto: 2 로 루프백]" --&gt; S2
+    S3 -- "참 (목표 3회 완료)&lt;br&gt;[Next Step: 4 로 정상 탈출]" --&gt; S4
+    S4 --&gt; EndNode
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="B14" s="28" t="inlineStr">
+        <is>
+          <t>│</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="B15" s="28" t="inlineStr">
+        <is>
+          <t>▼</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="26" customHeight="1">
+      <c r="B16" s="26" t="inlineStr">
+        <is>
+          <t>▶ [Step 2] 퍼지 가스 가압 (루프 시작점) | 10초 유지 (VN1=O, PNV=O / Alarm Goto 복귀 지점)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="B17" s="28" t="inlineStr">
+        <is>
+          <t>│</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="B18" s="28" t="inlineStr">
+        <is>
+          <t>▼</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="26" customHeight="1">
+      <c r="B19" s="31" t="inlineStr">
+        <is>
+          <t>◆ [Step 3] 배기 진행 및 반복 판정 | 15초 배기 후 판정: 진행횟수 &gt;= 3 ?</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="B20" s="28" t="inlineStr">
+        <is>
+          <t>├─ [거짓: 1~2회 미달] ➔ Alarm Goto 2로 재진입 (▲ Step 2 Loop-back)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="B21" s="28" t="inlineStr">
+        <is>
+          <t>└─ [참: 3회 완료] ➔ Next Step 4로 정상 탈출 (▼ Step 4 진행)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="26" customHeight="1">
+      <c r="B22" s="26" t="inlineStr">
+        <is>
+          <t>▶ [Step 4] 3회 반복 완료 및 정상 종료 | 5초 대기 (전 밸브 Close)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="B23" s="28" t="inlineStr">
+        <is>
+          <t>│</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="B24" s="28" t="inlineStr">
+        <is>
+          <t>▼</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="26" customHeight="1">
+      <c r="B25" s="29" t="inlineStr">
+        <is>
+          <t>★ [공정 정상 완료] | 3회 퍼지 사이클 완료</t>
+        </is>
+      </c>
+    </row>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="23">
+    <mergeCell ref="M3:Y3"/>
+    <mergeCell ref="B14:J14"/>
+    <mergeCell ref="B17:J17"/>
+    <mergeCell ref="B23:J23"/>
+    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="B13:J13"/>
+    <mergeCell ref="A11:AF11"/>
     <mergeCell ref="A2:L2"/>
+    <mergeCell ref="B19:J19"/>
     <mergeCell ref="A1:AF1"/>
-    <mergeCell ref="M3:Y3"/>
+    <mergeCell ref="M2:AF2"/>
+    <mergeCell ref="B24:J24"/>
+    <mergeCell ref="B15:J15"/>
+    <mergeCell ref="A12:K12"/>
+    <mergeCell ref="M13:AF33"/>
+    <mergeCell ref="B20:J20"/>
+    <mergeCell ref="M12:AF12"/>
+    <mergeCell ref="B16:J16"/>
+    <mergeCell ref="B25:J25"/>
+    <mergeCell ref="B22:J22"/>
     <mergeCell ref="Z3:AF3"/>
-    <mergeCell ref="M2:AF2"/>
-    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="B18:J18"/>
+    <mergeCell ref="B21:J21"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
@@ -4519,7 +5312,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF9"/>
+  <dimension ref="A1:AF36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -4826,7 +5619,7 @@
           <t>0.1</t>
         </is>
       </c>
-      <c r="AC5" s="24" t="inlineStr">
+      <c r="AC5" s="30" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -4940,7 +5733,9 @@
           <t>자동</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="n">
+        <v>99</v>
+      </c>
       <c r="I7" s="5" t="n">
         <v>99</v>
       </c>
@@ -5135,14 +5930,178 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12" ht="28" customHeight="1">
+      <c r="A12" s="24" t="inlineStr">
+        <is>
+          <t>📊 [공정 시퀀스 플로우차트 - 비주얼 블록 다이어그램 &amp; 공식 Mermaid 기법]</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>🎨 비주얼 공정 흐름도 (Visual Step Flowchart)</t>
+        </is>
+      </c>
+      <c r="M13" s="25" t="inlineStr">
+        <is>
+          <t>📜 공식 Mermaid 기법 소스 코드 (flowchart TD - 복사용)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="26" customHeight="1">
+      <c r="B14" s="26" t="inlineStr">
+        <is>
+          <t>▶ [Step 1] 배관 시험 진공 배기 | 30초 배기 (HPV=O, PNV=O / Early Pass Y)</t>
+        </is>
+      </c>
+      <c r="M14" s="27" t="inlineStr">
+        <is>
+          <t>```mermaid
+flowchart TD
+    classDef startNode fill:#1e40af,stroke:#1e3a8a,color:#fff,font-weight:bold
+    classDef procNode fill:#eff6ff,stroke:#3b82f6,color:#1e3a8a,font-weight:bold
+    classDef condNode fill:#fef3c7,stroke:#f59e0b,color:#b45309,font-weight:bold
+    classDef passNode fill:#d1fae5,stroke:#10b981,color:#047857,font-weight:bold
+    classDef alarmNode fill:#fee2e2,stroke:#ef4444,color:#b91c1c,font-weight:bold
+    Start(["[공정 시작] 예제6_누출시험"]):::startNode
+    S1["[Step 1] 배관 시험 진공 배기 (30초)&lt;br&gt;• HPV=O, PNV=O"]:::procNode
+    S2["[Step 2] 배관 밀폐 &amp; 초기압력 캡처 (5초)&lt;br&gt;• 전 밸브 Close&lt;br&gt;• Cycle: CAPTURE:VPT_{side} (P0 저장)"]:::procNode
+    S3{"[Step 3] 정밀 누출 감시 (60초)&lt;br&gt;감시: VPT:CAPOFFSET &lt;= 0.05 Torr"}:::condNode
+    S4["[Step 4] 누출 시험 합격 및 완료 (5초)&lt;br&gt;• 배관 건전성 통과 완료"]:::procNode
+    S99["[Step 99] 비상 정지 및 경보 (Alarm Seq 1)&lt;br&gt;• 허용치 초과 누출 발생!"]:::alarmNode
+    EndNode(["[공정 완료]"]):::passNode
+    Start --&gt; S1
+    S1 --&gt; S2
+    S2 --&gt; S3
+    S3 -- "변동량 &lt;= 0.05 Torr&lt;br&gt;(누출 없음 / 합격)" --&gt; S4
+    S3 -- "변동량 &gt; 0.05 Torr&lt;br&gt;(누출 발생 / Alarm Goto 99)" --&gt; S99
+    S4 --&gt; EndNode
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="B15" s="28" t="inlineStr">
+        <is>
+          <t>│</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="B16" s="28" t="inlineStr">
+        <is>
+          <t>▼</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="26" customHeight="1">
+      <c r="B17" s="26" t="inlineStr">
+        <is>
+          <t>▶ [Step 2] 배관 밀폐 및 초기값 캡처 | 5초 대기 (Cycle: CAPTURE:VPT_{side} ➔ 기준압력 P0 저장)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="B18" s="28" t="inlineStr">
+        <is>
+          <t>│</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="B19" s="28" t="inlineStr">
+        <is>
+          <t>▼</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="26" customHeight="1">
+      <c r="B20" s="31" t="inlineStr">
+        <is>
+          <t>◆ [Step 3] 정밀 감압 누출 감시 | 60초 감시: VPT_{side}:CAPOFFSET &lt;= 0.05 Torr ?</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="B21" s="28" t="inlineStr">
+        <is>
+          <t>├─ [참: 상승량 &lt;= 0.05 Torr] ➔ ★ 합격 (Step 4 진행)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="B22" s="28" t="inlineStr">
+        <is>
+          <t>└─ [거짓: 허용치 초과 누출] ➔ ▲ 비상 알람 발생 (Alarm Goto: 99)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="26" customHeight="1">
+      <c r="B23" s="26" t="inlineStr">
+        <is>
+          <t>▶ [Step 4] 누출 시험 합격 및 완료 | 5초 대기 (배관 건전성 확인 완료)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="B24" s="28" t="inlineStr">
+        <is>
+          <t>│</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="B25" s="28" t="inlineStr">
+        <is>
+          <t>▼</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="26" customHeight="1">
+      <c r="B26" s="29" t="inlineStr">
+        <is>
+          <t>★ [공정 정상 완료] | 누출 시험 통과 후 공정 종료</t>
+        </is>
+      </c>
+    </row>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="23">
+    <mergeCell ref="M3:Y3"/>
+    <mergeCell ref="B14:J14"/>
+    <mergeCell ref="B17:J17"/>
+    <mergeCell ref="B23:J23"/>
+    <mergeCell ref="A3:L3"/>
     <mergeCell ref="A2:L2"/>
+    <mergeCell ref="B19:J19"/>
     <mergeCell ref="A1:AF1"/>
-    <mergeCell ref="M3:Y3"/>
+    <mergeCell ref="M2:AF2"/>
+    <mergeCell ref="B24:J24"/>
+    <mergeCell ref="B15:J15"/>
+    <mergeCell ref="B20:J20"/>
+    <mergeCell ref="M13:AF13"/>
+    <mergeCell ref="B26:J26"/>
+    <mergeCell ref="A12:AF12"/>
+    <mergeCell ref="B16:J16"/>
+    <mergeCell ref="B25:J25"/>
+    <mergeCell ref="M14:AF36"/>
+    <mergeCell ref="B22:J22"/>
     <mergeCell ref="Z3:AF3"/>
-    <mergeCell ref="M2:AF2"/>
-    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="B18:J18"/>
+    <mergeCell ref="A13:K13"/>
+    <mergeCell ref="B21:J21"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
@@ -5157,7 +6116,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF13"/>
+  <dimension ref="A1:AF49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -5628,7 +6587,7 @@
           <t>0.5</t>
         </is>
       </c>
-      <c r="AC7" s="24" t="inlineStr">
+      <c r="AC7" s="30" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -6121,14 +7080,280 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16" ht="28" customHeight="1">
+      <c r="A16" s="24" t="inlineStr">
+        <is>
+          <t>📊 [공정 시퀀스 플로우차트 - 비주얼 블록 다이어그램 &amp; 공식 Mermaid 기법]</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>🎨 비주얼 공정 흐름도 (Visual Step Flowchart)</t>
+        </is>
+      </c>
+      <c r="M17" s="25" t="inlineStr">
+        <is>
+          <t>📜 공식 Mermaid 기법 소스 코드 (flowchart TD - 복사용)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="26" customHeight="1">
+      <c r="B18" s="26" t="inlineStr">
+        <is>
+          <t>▶ [Step 1] 전 밸브 안전 초기화 | 5초 대기 (전 밸브 Close)</t>
+        </is>
+      </c>
+      <c r="M18" s="27" t="inlineStr">
+        <is>
+          <t>```mermaid
+flowchart TD
+    classDef startNode fill:#1e40af,stroke:#1e3a8a,color:#fff,font-weight:bold
+    classDef procNode fill:#eff6ff,stroke:#3b82f6,color:#1e3a8a,font-weight:bold
+    classDef condNode fill:#fef3c7,stroke:#f59e0b,color:#b45309,font-weight:bold
+    classDef passNode fill:#d1fae5,stroke:#10b981,color:#047857,font-weight:bold
+    classDef alarmNode fill:#fee2e2,stroke:#ef4444,color:#b91c1c,font-weight:bold
+    Start(["[공정 시작] Bypass_v1 종합 실전"]):::startNode
+    S1["[Step 1] 전 밸브 안전 초기화 (5초)"]:::procNode
+    S2["[Step 2] 1차 질소 공급 및 퍼지 (20초)&lt;br&gt;• VN1=O, PNV=O"]:::procNode
+    S3{"[Step 3] 2차 진공 배기 120초&lt;br&gt;감시: VPT &lt;= 0.5 Torr (조기통과 Y)"}:::condNode
+    S4{"[Step 4] 작업자 육안 확인&lt;br&gt;• 진행방식 = 확인 (ACK)"}:::condNode
+    S5["[Step 5] 순차 지연 개방 (15초)&lt;br&gt;• VN2(0s) ➔ LPV(2s) ➔ HPIV(4s)"]:::procNode
+    S6["[Step 6] 3회 반복 퍼지 - 가압 (10초)&lt;br&gt;★ 루프 시작점 (Alarm Goto 목적지)"]:::procNode
+    S7{"[Step 7] 배기 및 3회 반복 판정 (15초)&lt;br&gt;판정: 진행횟수 &gt;= 3 ?"}:::condNode
+    S8["[Step 8] 전 밸브 Close 및 완료 (5초)"]:::procNode
+    S99["[Step 99] 비상 알람 조치 스텝 (Alarm Seq 1)"]:::alarmNode
+    EndNode(["[Bypass 전 공정 정상 완료]"]):::passNode
+    Start --&gt; S1
+    S1 --&gt; S2
+    S2 --&gt; S3
+    S3 -- "0.5 Torr 도달&lt;br&gt;(조기통과!)" --&gt; S4
+    S3 -- "120초 미도달&lt;br&gt;[Alarm Goto: 99]" --&gt; S99
+    S4 -- "작업자 [확인] 클릭" --&gt; S5
+    S5 --&gt; S6
+    S6 --&gt; S7
+    S7 -- "거짓 (1~2회차 미달)&lt;br&gt;[Alarm Goto: 6 으로 루프백]" --&gt; S6
+    S7 -- "참 (3회 완료)&lt;br&gt;[Next Step: 8 로 정상 탈출]" --&gt; S8
+    S8 --&gt; EndNode
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="B19" s="28" t="inlineStr">
+        <is>
+          <t>│</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="B20" s="28" t="inlineStr">
+        <is>
+          <t>▼</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="26" customHeight="1">
+      <c r="B21" s="26" t="inlineStr">
+        <is>
+          <t>▶ [Step 2] 1차 질소 공급 및 퍼지 | 20초 유지 (VN1=O, PNV=O)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="B22" s="28" t="inlineStr">
+        <is>
+          <t>│</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="B23" s="28" t="inlineStr">
+        <is>
+          <t>▼</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="26" customHeight="1">
+      <c r="B24" s="31" t="inlineStr">
+        <is>
+          <t>◆ [Step 3] 2차 진공 배기 (조기통과 Y) | 120초 (VPT &lt;= 0.5 Torr 시 즉시 패스, 초과 시 Step 99 알람)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="B25" s="28" t="inlineStr">
+        <is>
+          <t>│</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="B26" s="28" t="inlineStr">
+        <is>
+          <t>▼</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="26" customHeight="1">
+      <c r="B27" s="31" t="inlineStr">
+        <is>
+          <t>◆ [Step 4] 작업자 육안 확인 (ACK 대기) | 진행방식 = 확인 (작업자 [확인] 클릭 시까지 대기)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="B28" s="28" t="inlineStr">
+        <is>
+          <t>│</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="B29" s="28" t="inlineStr">
+        <is>
+          <t>▼</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="26" customHeight="1">
+      <c r="B30" s="26" t="inlineStr">
+        <is>
+          <t>▶ [Step 5] 밸브 순차 지연 개폐 제어 | 15초 (VN2=0s ➔ LPV=2s ➔ HPIV=4s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="B31" s="28" t="inlineStr">
+        <is>
+          <t>│</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="22" customHeight="1">
+      <c r="B32" s="28" t="inlineStr">
+        <is>
+          <t>▼</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="26" customHeight="1">
+      <c r="B33" s="26" t="inlineStr">
+        <is>
+          <t>▶ [Step 6] 3회 반복 퍼지 - 가압 | 10초 (루프 시작점 / Alarm Goto 목적지)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="22" customHeight="1">
+      <c r="B34" s="28" t="inlineStr">
+        <is>
+          <t>│</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="22" customHeight="1">
+      <c r="B35" s="28" t="inlineStr">
+        <is>
+          <t>▼</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="26" customHeight="1">
+      <c r="B36" s="31" t="inlineStr">
+        <is>
+          <t>◆ [Step 7] 3회 반복 퍼지 - 배기 및 판정 | 15초 배기 후 판정: 진행횟수 &gt;= 3 ?</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="22" customHeight="1">
+      <c r="B37" s="28" t="inlineStr">
+        <is>
+          <t>├─ [거짓: 1~2회 미달] ➔ Alarm Goto 6 으로 재진입 (▲ Step 6 Loop)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="22" customHeight="1">
+      <c r="B38" s="28" t="inlineStr">
+        <is>
+          <t>└─ [참: 3회 완료] ➔ Next Step 8 로 정상 탈출 (▼ Step 8 진행)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="26" customHeight="1">
+      <c r="B39" s="26" t="inlineStr">
+        <is>
+          <t>▶ [Step 8] 공정 완료 및 전 밸브 Close | 5초 대기</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="22" customHeight="1">
+      <c r="B40" s="28" t="inlineStr">
+        <is>
+          <t>│</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="22" customHeight="1">
+      <c r="B41" s="28" t="inlineStr">
+        <is>
+          <t>▼</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="26" customHeight="1">
+      <c r="B42" s="29" t="inlineStr">
+        <is>
+          <t>★ [Bypass 종합 공정 정상 완료] | 모든 단계 완벽 수행 완료</t>
+        </is>
+      </c>
+    </row>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="35">
+    <mergeCell ref="B42:J42"/>
+    <mergeCell ref="M3:Y3"/>
+    <mergeCell ref="B23:J23"/>
+    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="B38:J38"/>
+    <mergeCell ref="B29:J29"/>
     <mergeCell ref="A2:L2"/>
+    <mergeCell ref="B19:J19"/>
+    <mergeCell ref="B34:J34"/>
+    <mergeCell ref="B37:J37"/>
     <mergeCell ref="A1:AF1"/>
-    <mergeCell ref="M3:Y3"/>
+    <mergeCell ref="B28:J28"/>
+    <mergeCell ref="B40:J40"/>
+    <mergeCell ref="M2:AF2"/>
+    <mergeCell ref="B24:J24"/>
+    <mergeCell ref="A16:AF16"/>
+    <mergeCell ref="B30:J30"/>
+    <mergeCell ref="B33:J33"/>
+    <mergeCell ref="B20:J20"/>
+    <mergeCell ref="M18:AF49"/>
+    <mergeCell ref="B36:J36"/>
+    <mergeCell ref="B32:J32"/>
+    <mergeCell ref="B26:J26"/>
+    <mergeCell ref="B41:J41"/>
+    <mergeCell ref="B35:J35"/>
+    <mergeCell ref="A17:K17"/>
+    <mergeCell ref="B25:J25"/>
+    <mergeCell ref="M17:AF17"/>
+    <mergeCell ref="B22:J22"/>
     <mergeCell ref="Z3:AF3"/>
-    <mergeCell ref="M2:AF2"/>
-    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="B31:J31"/>
+    <mergeCell ref="B18:J18"/>
+    <mergeCell ref="B27:J27"/>
+    <mergeCell ref="B39:J39"/>
+    <mergeCell ref="B21:J21"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>

</xml_diff>